<commit_message>
Statistcal and Math function
</commit_message>
<xml_diff>
--- a/2_Formulas_Functions/3_Logical_Functions.xlsx
+++ b/2_Formulas_Functions/3_Logical_Functions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\python\Excel_Data_Analytics\2_Formulas_Functions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07BB909D-E12F-4DC4-A621-1A6646D598E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FF610E1-55A2-467C-840F-38C05DA74006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{8CC555B5-3E06-43B6-9E5B-C0A1D3498DA4}"/>
   </bookViews>
@@ -1484,7 +1484,7 @@
         <v>0</v>
       </c>
       <c r="L4" s="19" t="b">
-        <f t="shared" ref="L3:L12" si="7">$C$15&lt;=C4</f>
+        <f t="shared" ref="L4:L12" si="7">$C$15&lt;=C4</f>
         <v>0</v>
       </c>
       <c r="M4" s="19" t="b">
@@ -2762,15 +2762,17 @@
   <cols>
     <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.140625" customWidth="1"/>
-    <col min="3" max="3" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="38.140625" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="79.7109375" customWidth="1"/>
+    <col min="10" max="10" width="79.42578125" hidden="1" customWidth="1"/>
     <col min="11" max="18" width="16.140625" customWidth="1"/>
+    <col min="19" max="19" width="13.85546875" customWidth="1"/>
+    <col min="20" max="20" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -2880,6 +2882,14 @@
         <f>OR($A2 =$K$1, $A2 = $L$1)</f>
         <v>0</v>
       </c>
+      <c r="P2" t="str">
+        <f>IF(OR($A2=$K$1, $A2=$L$1),"Role Desired","Not Desired")</f>
+        <v>Not Desired</v>
+      </c>
+      <c r="Q2" t="str">
+        <f>IF($H2 &gt; 85000, "Salary &gt; 85k","Salary Low")</f>
+        <v>Salary &gt; 85k</v>
+      </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="27" t="s">
@@ -2932,6 +2942,14 @@
         <f t="shared" ref="O3:O21" si="4">OR($A3 =$K$1, $A3 = $L$1)</f>
         <v>1</v>
       </c>
+      <c r="P3" t="str">
+        <f>IF(OR($A3=$K$1, $A3=$L$1),"Role Desired","Not Desired")</f>
+        <v>Role Desired</v>
+      </c>
+      <c r="Q3" t="str">
+        <f t="shared" ref="Q3:Q21" si="5">IF($H3 &gt; 85000, "Salary &gt; 85k","Salary Low")</f>
+        <v>Salary Low</v>
+      </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
@@ -2982,6 +3000,14 @@
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
+      <c r="P4" t="str">
+        <f t="shared" ref="P3:P21" si="6">IF(OR($A4=$K$1, $A4=$L$1),"Role Desired","Not Desired")</f>
+        <v>Role Desired</v>
+      </c>
+      <c r="Q4" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary Low</v>
+      </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
@@ -3032,6 +3058,14 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="P5" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Desired</v>
+      </c>
+      <c r="Q5" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary Low</v>
+      </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
@@ -3082,6 +3116,14 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="P6" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Desired</v>
+      </c>
+      <c r="Q6" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary Low</v>
+      </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="27" t="s">
@@ -3132,6 +3174,14 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="P7" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Desired</v>
+      </c>
+      <c r="Q7" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary Low</v>
+      </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
@@ -3179,8 +3229,16 @@
         <v>0</v>
       </c>
       <c r="O8" t="b">
-        <f t="shared" si="4"/>
-        <v>1</v>
+        <f>OR($A8 =$K$1, $A8 = $L$1)</f>
+        <v>1</v>
+      </c>
+      <c r="P8" t="str">
+        <f t="shared" si="6"/>
+        <v>Role Desired</v>
+      </c>
+      <c r="Q8" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary Low</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
@@ -3234,6 +3292,14 @@
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
+      <c r="P9" t="str">
+        <f t="shared" si="6"/>
+        <v>Role Desired</v>
+      </c>
+      <c r="Q9" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary &gt; 85k</v>
+      </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
@@ -3284,6 +3350,14 @@
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
+      <c r="P10" t="str">
+        <f t="shared" si="6"/>
+        <v>Role Desired</v>
+      </c>
+      <c r="Q10" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary Low</v>
+      </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
@@ -3336,6 +3410,14 @@
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
+      <c r="P11" t="str">
+        <f t="shared" si="6"/>
+        <v>Role Desired</v>
+      </c>
+      <c r="Q11" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary &gt; 85k</v>
+      </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
@@ -3388,6 +3470,14 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="P12" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Desired</v>
+      </c>
+      <c r="Q12" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary &gt; 85k</v>
+      </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
@@ -3440,6 +3530,14 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="P13" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Desired</v>
+      </c>
+      <c r="Q13" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary &gt; 85k</v>
+      </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
@@ -3492,6 +3590,14 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="P14" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Desired</v>
+      </c>
+      <c r="Q14" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary &gt; 85k</v>
+      </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
@@ -3544,6 +3650,14 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="P15" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Desired</v>
+      </c>
+      <c r="Q15" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary Low</v>
+      </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
@@ -3596,8 +3710,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P16" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Desired</v>
+      </c>
+      <c r="Q16" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary &gt; 85k</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
         <v>4</v>
       </c>
@@ -3648,8 +3770,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P17" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Desired</v>
+      </c>
+      <c r="Q17" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary &gt; 85k</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
         <v>123</v>
       </c>
@@ -3698,8 +3828,16 @@
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P18" t="str">
+        <f t="shared" si="6"/>
+        <v>Role Desired</v>
+      </c>
+      <c r="Q18" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary Low</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
         <v>0</v>
       </c>
@@ -3750,8 +3888,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P19" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Desired</v>
+      </c>
+      <c r="Q19" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary &gt; 85k</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
         <v>0</v>
       </c>
@@ -3800,8 +3946,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P20" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Desired</v>
+      </c>
+      <c r="Q20" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary Low</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
         <v>123</v>
       </c>
@@ -3851,6 +4005,14 @@
       <c r="O21" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
+      </c>
+      <c r="P21" t="str">
+        <f t="shared" si="6"/>
+        <v>Role Desired</v>
+      </c>
+      <c r="Q21" t="str">
+        <f t="shared" si="5"/>
+        <v>Salary &gt; 85k</v>
       </c>
     </row>
   </sheetData>
@@ -4002,9 +4164,9 @@
         <f>IF($H2&gt;$Q$1, "Salary &gt; 85K", "Salary Low")</f>
         <v>Salary &gt; 85K</v>
       </c>
-      <c r="R2" t="str" cm="1">
-        <f t="array" ref="R2">_xlfn.IFS(H2="", "No Data", H2&gt;=$Q$1, "Salary &gt; 85K", TRUE, "Salary Low")</f>
-        <v>Salary &gt; 85K</v>
+      <c r="R2" t="e">
+        <f ca="1">_xlfn.IFS(H2="", "No Data", H2&gt;=$Q$1, "Salary &gt; 85K", TRUE, "Salary Low")</f>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="3" spans="1:18 16384:16384" x14ac:dyDescent="0.25">
@@ -4066,9 +4228,9 @@
         <f t="shared" ref="Q3:Q21" si="5">IF($H3&gt;$Q$1, "Salary &gt; 85K", "Salary Low")</f>
         <v>Salary Low</v>
       </c>
-      <c r="R3" t="str" cm="1">
-        <f t="array" ref="R3">_xlfn.IFS(H3="", "No Data", H3&gt;=$Q$1, "Salary &gt; 85K", TRUE, "Salary Low")</f>
-        <v>Salary Low</v>
+      <c r="R3" t="e">
+        <f ca="1">_xlfn.IFS(H3="", "No Data", H3&gt;=$Q$1, "Salary &gt; 85K", TRUE, "Salary Low")</f>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="4" spans="1:18 16384:16384" x14ac:dyDescent="0.25">
@@ -4113,7 +4275,7 @@
         <v>Role Desired</v>
       </c>
       <c r="N4" t="b">
-        <f t="shared" ref="N3:N21" si="6">AND($A4=$K$1, $A4=$L$1)</f>
+        <f t="shared" ref="N4:N21" si="6">AND($A4=$K$1, $A4=$L$1)</f>
         <v>0</v>
       </c>
       <c r="O4" t="b">
@@ -4128,9 +4290,9 @@
         <f t="shared" si="5"/>
         <v>Salary Low</v>
       </c>
-      <c r="R4" t="str" cm="1">
-        <f t="array" ref="R4">_xlfn.IFS(H4="", "No Data", H4&gt;=$Q$1, "Salary &gt; 85K", TRUE, "Salary Low")</f>
-        <v>No Data</v>
+      <c r="R4" t="e">
+        <f ca="1">_xlfn.IFS(H4="", "No Data", H4&gt;=$Q$1, "Salary &gt; 85K", TRUE, "Salary Low")</f>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="5" spans="1:18 16384:16384" x14ac:dyDescent="0.25">
@@ -4190,9 +4352,9 @@
         <f t="shared" si="5"/>
         <v>Salary Low</v>
       </c>
-      <c r="R5" t="str" cm="1">
-        <f t="array" ref="R5">_xlfn.IFS(H5="", "No Data", H5&gt;=$Q$1, "Salary &gt; 85K", TRUE, "Salary Low")</f>
-        <v>No Data</v>
+      <c r="R5" t="e">
+        <f ca="1">IFS(H5="", "No Data", H5&gt;=$Q$1, "Salary &gt; 85K", TRUE, "Salary Low")</f>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="6" spans="1:18 16384:16384" x14ac:dyDescent="0.25">

</xml_diff>